<commit_message>
Fix label truncation in invoice/quote samples; add listing preview image
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y6nZA9prevJ6RsNJnLc7d4
</commit_message>
<xml_diff>
--- a/sales/samples/invoice-template.xlsx
+++ b/sales/samples/invoice-template.xlsx
@@ -507,8 +507,8 @@
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1097,18 +1097,18 @@
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="A35:E35"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="A38:E38"/>
     <mergeCell ref="B43:F45"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="A33:E33"/>
-    <mergeCell ref="A40:E40"/>
+    <mergeCell ref="A41:E41"/>
     <mergeCell ref="B9:D9"/>
-    <mergeCell ref="A41:E41"/>
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="A36:E36"/>
-    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A40:E40"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="D12:D31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>